<commit_message>
data(week 20): correct channel names in Tonor/WM other_channels + re-run
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/sales/Week 20/Tonor/other_channels.xlsx
+++ b/data/raw/sales/Week 20/Tonor/other_channels.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\sales\Week 20\Tonor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C59D34A0-BB4F-45C7-B061-50E72A0B04F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63DD7A05-A721-40FE-9062-5BAF1A3CBAAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="1p" sheetId="13" r:id="rId1"/>
+    <sheet name="1p Sales" sheetId="13" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>